<commit_message>
refactor the data extraction and chrome driver fix code
</commit_message>
<xml_diff>
--- a/coach_numbers.xlsx
+++ b/coach_numbers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ANUP JS LEARNING\automate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ANUP JS LEARNING\GIT UPDATED SOFTWARE\CMM-data-extractor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A5831F-BC20-4D87-BF6C-C2707A71FB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A182422-3417-4F71-A1DB-665DC1B88B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="0" windowWidth="12980" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="0" windowWidth="12980" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -145,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -157,9 +157,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -167,6 +164,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,229 +467,163 @@
       </c>
     </row>
     <row r="2" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="5">
-        <v>126085</v>
+      <c r="A2" s="8">
+        <v>201504</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="6">
-        <v>221390</v>
+      <c r="A3" s="9">
+        <v>193915</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="6">
-        <v>221394</v>
+      <c r="A4" s="9">
+        <v>31080</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="6">
-        <v>221402</v>
+      <c r="A5" s="9">
+        <v>41010</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="6">
-        <v>223250</v>
+      <c r="A6" s="9">
+        <v>196188</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="6">
-        <v>223758</v>
+      <c r="A7" s="9">
+        <v>169272</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="6">
-        <v>191478</v>
+      <c r="A8" s="9">
+        <v>974388</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="6">
-        <v>191555</v>
+      <c r="A9" s="9">
+        <v>28760</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="6">
-        <v>223231</v>
+      <c r="A10" s="9">
+        <v>194798</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="6">
-        <v>223248</v>
+      <c r="A11" s="9">
+        <v>41244</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="6">
-        <v>223266</v>
+      <c r="A12" s="10">
+        <v>196182</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="6">
-        <v>101348</v>
+      <c r="A13" s="9">
+        <v>193891</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="6">
-        <v>67231</v>
-      </c>
+      <c r="A14" s="5"/>
     </row>
     <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="6">
-        <v>47077</v>
-      </c>
+      <c r="A15" s="5"/>
     </row>
     <row r="16" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="6">
-        <v>126095</v>
-      </c>
+      <c r="A16" s="5"/>
     </row>
     <row r="17" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="6">
-        <v>126125</v>
-      </c>
+      <c r="A17" s="5"/>
     </row>
     <row r="18" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="6">
-        <v>126065</v>
-      </c>
+      <c r="A18" s="5"/>
     </row>
     <row r="19" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="6">
-        <v>182380</v>
-      </c>
+      <c r="A19" s="5"/>
     </row>
     <row r="20" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="6">
-        <v>181654</v>
-      </c>
+      <c r="A20" s="5"/>
     </row>
     <row r="21" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="6">
-        <v>223262</v>
-      </c>
+      <c r="A21" s="5"/>
     </row>
     <row r="22" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="6">
-        <v>221333</v>
-      </c>
+      <c r="A22" s="5"/>
     </row>
     <row r="23" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="6">
-        <v>224104</v>
-      </c>
+      <c r="A23" s="5"/>
     </row>
     <row r="24" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="6">
-        <v>224467</v>
-      </c>
+      <c r="A24" s="5"/>
     </row>
     <row r="25" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="6">
-        <v>222094</v>
-      </c>
+      <c r="A25" s="5"/>
     </row>
     <row r="26" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="6">
-        <v>193874</v>
-      </c>
+      <c r="A26" s="5"/>
     </row>
     <row r="27" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="6">
-        <v>223763</v>
-      </c>
+      <c r="A27" s="5"/>
     </row>
     <row r="28" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="7">
-        <v>111535</v>
-      </c>
+      <c r="A28" s="6"/>
     </row>
     <row r="29" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="7">
-        <v>182382</v>
-      </c>
+      <c r="A29" s="6"/>
     </row>
     <row r="30" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="7">
-        <v>121178</v>
-      </c>
+      <c r="A30" s="6"/>
     </row>
     <row r="31" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="7">
-        <v>191543</v>
-      </c>
+      <c r="A31" s="6"/>
     </row>
     <row r="32" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="7">
-        <v>126145</v>
-      </c>
+      <c r="A32" s="6"/>
     </row>
     <row r="33" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="7">
-        <v>193924</v>
-      </c>
+      <c r="A33" s="6"/>
     </row>
     <row r="34" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="8">
-        <v>151330</v>
-      </c>
+      <c r="A34" s="7"/>
     </row>
     <row r="35" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="7">
-        <v>164512</v>
-      </c>
+      <c r="A35" s="6"/>
     </row>
     <row r="36" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="7">
-        <v>181652</v>
-      </c>
+      <c r="A36" s="6"/>
     </row>
     <row r="37" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="7">
-        <v>221400</v>
-      </c>
+      <c r="A37" s="6"/>
     </row>
     <row r="38" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="7">
-        <v>224108</v>
-      </c>
+      <c r="A38" s="6"/>
     </row>
     <row r="39" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="7">
-        <v>122234</v>
-      </c>
+      <c r="A39" s="6"/>
     </row>
     <row r="40" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="7">
-        <v>131187</v>
-      </c>
+      <c r="A40" s="6"/>
     </row>
     <row r="41" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="7">
-        <v>223264</v>
-      </c>
+      <c r="A41" s="6"/>
     </row>
     <row r="42" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="7">
-        <v>191531</v>
-      </c>
+      <c r="A42" s="6"/>
     </row>
     <row r="43" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="7">
-        <v>221403</v>
-      </c>
+      <c r="A43" s="6"/>
     </row>
     <row r="44" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="7">
-        <v>224778</v>
-      </c>
+      <c r="A44" s="6"/>
     </row>
     <row r="45" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A45" s="7">
-        <v>223759</v>
-      </c>
+      <c r="A45" s="6"/>
     </row>
     <row r="46" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A46" s="7">
-        <v>225928</v>
-      </c>
+      <c r="A46" s="6"/>
     </row>
     <row r="47" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="2"/>

</xml_diff>

<commit_message>
final done - NEW COMMISSIONED project
</commit_message>
<xml_diff>
--- a/coach_numbers.xlsx
+++ b/coach_numbers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ANUP JS LEARNING\GIT UPDATED SOFTWARE\CMM-data-extractor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A182422-3417-4F71-A1DB-665DC1B88B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED24B54A-3BB6-4FE4-9B63-70CE52BE9A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="0" windowWidth="12980" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -478,68 +478,64 @@
     </row>
     <row r="4" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="9">
-        <v>31080</v>
+        <v>259076</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="9">
-        <v>41010</v>
+        <v>169272</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="9">
-        <v>196188</v>
+        <v>974388</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="9">
-        <v>169272</v>
+        <v>28760</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="9">
-        <v>974388</v>
+        <v>194798</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="9">
-        <v>28760</v>
+        <v>41244</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="9">
-        <v>194798</v>
+      <c r="A10" s="10">
+        <v>196182</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="9">
-        <v>41244</v>
+        <v>193891</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="10">
-        <v>196182</v>
-      </c>
+      <c r="A12" s="9"/>
     </row>
     <row r="13" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="9">
-        <v>193891</v>
-      </c>
+      <c r="A13" s="9"/>
     </row>
     <row r="14" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="5"/>
+      <c r="A14" s="9"/>
     </row>
     <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="5"/>
+      <c r="A15" s="9"/>
     </row>
     <row r="16" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="5"/>
+      <c r="A16" s="9"/>
     </row>
     <row r="17" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="5"/>
+      <c r="A17" s="9"/>
     </row>
     <row r="18" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="5"/>
+      <c r="A18" s="9"/>
     </row>
     <row r="19" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="5"/>

</xml_diff>